<commit_message>
Fix: strip stray merge-conflict markers from live.js; rebuild xlsx
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/earnings-data.xlsx
+++ b/earnings-data.xlsx
@@ -12921,7 +12921,7 @@
         <v>0.193</v>
       </c>
       <c r="G162" s="6" t="n">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="H162" s="7" t="inlineStr">
         <is>
@@ -12930,7 +12930,7 @@
       </c>
       <c r="I162" s="3" t="inlineStr">
         <is>
-          <t>Oct 20 (est)</t>
+          <t>Oct 22 (est)</t>
         </is>
       </c>
       <c r="J162" s="3" t="inlineStr"/>
@@ -20718,7 +20718,7 @@
       </c>
       <c r="I282" s="3" t="inlineStr">
         <is>
-          <t>Jul 29 (est)  ·  Oct 28 (est)</t>
+          <t>Jul 29 (est)  ·  Nov 04 (est)</t>
         </is>
       </c>
       <c r="J282" s="3" t="inlineStr"/>
@@ -34135,17 +34135,17 @@
       </c>
       <c r="C306" s="30" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="D306" s="29" t="inlineStr">
         <is>
-          <t>RTX Corp</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E306" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F306" s="29" t="inlineStr"/>
@@ -34157,21 +34157,21 @@
     </row>
     <row r="307">
       <c r="A307" s="28" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B307" s="29" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C307" s="30" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="D307" s="29" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Amphenol</t>
         </is>
       </c>
       <c r="E307" s="29" t="inlineStr">
@@ -34197,17 +34197,17 @@
       </c>
       <c r="C308" s="30" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>BSX</t>
         </is>
       </c>
       <c r="D308" s="29" t="inlineStr">
         <is>
-          <t>Amphenol</t>
+          <t>Boston Scientific</t>
         </is>
       </c>
       <c r="E308" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F308" s="29" t="inlineStr"/>
@@ -34228,17 +34228,17 @@
       </c>
       <c r="C309" s="30" t="inlineStr">
         <is>
-          <t>BSX</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="D309" s="29" t="inlineStr">
         <is>
-          <t>Boston Scientific</t>
+          <t>GE Vernova</t>
         </is>
       </c>
       <c r="E309" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F309" s="29" t="inlineStr"/>
@@ -34259,17 +34259,17 @@
       </c>
       <c r="C310" s="30" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="D310" s="29" t="inlineStr">
         <is>
-          <t>GE Vernova</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="E310" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F310" s="29" t="inlineStr"/>
@@ -34290,17 +34290,17 @@
       </c>
       <c r="C311" s="30" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>KMI</t>
         </is>
       </c>
       <c r="D311" s="29" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>Kinder Morgan</t>
         </is>
       </c>
       <c r="E311" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F311" s="29" t="inlineStr"/>
@@ -34321,17 +34321,17 @@
       </c>
       <c r="C312" s="30" t="inlineStr">
         <is>
-          <t>KMI</t>
+          <t>LII</t>
         </is>
       </c>
       <c r="D312" s="29" t="inlineStr">
         <is>
-          <t>Kinder Morgan</t>
+          <t>Lennox Intl</t>
         </is>
       </c>
       <c r="E312" s="29" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F312" s="29" t="inlineStr"/>
@@ -34352,17 +34352,17 @@
       </c>
       <c r="C313" s="30" t="inlineStr">
         <is>
-          <t>LII</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="D313" s="29" t="inlineStr">
         <is>
-          <t>Lennox Intl</t>
+          <t>Lam Research</t>
         </is>
       </c>
       <c r="E313" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F313" s="29" t="inlineStr"/>
@@ -34383,17 +34383,17 @@
       </c>
       <c r="C314" s="30" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>ORLY</t>
         </is>
       </c>
       <c r="D314" s="29" t="inlineStr">
         <is>
-          <t>Lam Research</t>
+          <t>O'Reilly Auto</t>
         </is>
       </c>
       <c r="E314" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="F314" s="29" t="inlineStr"/>
@@ -34414,17 +34414,17 @@
       </c>
       <c r="C315" s="30" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>PKG</t>
         </is>
       </c>
       <c r="D315" s="29" t="inlineStr">
         <is>
-          <t>O'Reilly Auto</t>
+          <t>Packaging Corp</t>
         </is>
       </c>
       <c r="E315" s="29" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F315" s="29" t="inlineStr"/>
@@ -34445,17 +34445,17 @@
       </c>
       <c r="C316" s="30" t="inlineStr">
         <is>
-          <t>PKG</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="D316" s="29" t="inlineStr">
         <is>
-          <t>Packaging Corp</t>
+          <t>SAP SE</t>
         </is>
       </c>
       <c r="E316" s="29" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F316" s="29" t="inlineStr"/>
@@ -34476,17 +34476,17 @@
       </c>
       <c r="C317" s="30" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>SEIC</t>
         </is>
       </c>
       <c r="D317" s="29" t="inlineStr">
         <is>
-          <t>SAP SE</t>
+          <t>SEI Investments</t>
         </is>
       </c>
       <c r="E317" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F317" s="29" t="inlineStr"/>
@@ -34507,17 +34507,17 @@
       </c>
       <c r="C318" s="30" t="inlineStr">
         <is>
-          <t>SEIC</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="D318" s="29" t="inlineStr">
         <is>
-          <t>SEI Investments</t>
+          <t>Thermo Fisher</t>
         </is>
       </c>
       <c r="E318" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F318" s="29" t="inlineStr"/>
@@ -34538,17 +34538,17 @@
       </c>
       <c r="C319" s="30" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="D319" s="29" t="inlineStr">
         <is>
-          <t>Thermo Fisher</t>
+          <t>Tesla</t>
         </is>
       </c>
       <c r="E319" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="F319" s="29" t="inlineStr"/>
@@ -34569,17 +34569,17 @@
       </c>
       <c r="C320" s="30" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="D320" s="29" t="inlineStr">
         <is>
-          <t>Tesla</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="E320" s="29" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F320" s="29" t="inlineStr"/>
@@ -34591,26 +34591,26 @@
     </row>
     <row r="321">
       <c r="A321" s="28" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B321" s="29" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C321" s="30" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="D321" s="29" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Baker Hughes</t>
         </is>
       </c>
       <c r="E321" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F321" s="29" t="inlineStr"/>
@@ -34631,17 +34631,17 @@
       </c>
       <c r="C322" s="30" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="D322" s="29" t="inlineStr">
         <is>
-          <t>Baker Hughes</t>
+          <t>Blackstone</t>
         </is>
       </c>
       <c r="E322" s="29" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F322" s="29" t="inlineStr"/>
@@ -34662,17 +34662,17 @@
       </c>
       <c r="C323" s="30" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>CBRE</t>
         </is>
       </c>
       <c r="D323" s="29" t="inlineStr">
         <is>
-          <t>Blackstone</t>
+          <t>CBRE Group</t>
         </is>
       </c>
       <c r="E323" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="F323" s="29" t="inlineStr"/>
@@ -34693,12 +34693,12 @@
       </c>
       <c r="C324" s="30" t="inlineStr">
         <is>
-          <t>CBRE</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="D324" s="29" t="inlineStr">
         <is>
-          <t>CBRE Group</t>
+          <t>Digital Realty</t>
         </is>
       </c>
       <c r="E324" s="29" t="inlineStr">
@@ -34724,17 +34724,17 @@
       </c>
       <c r="C325" s="30" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>DOW</t>
         </is>
       </c>
       <c r="D325" s="29" t="inlineStr">
         <is>
-          <t>Digital Realty</t>
+          <t>Dow</t>
         </is>
       </c>
       <c r="E325" s="29" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F325" s="29" t="inlineStr"/>
@@ -34755,12 +34755,12 @@
       </c>
       <c r="C326" s="30" t="inlineStr">
         <is>
-          <t>DOW</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="D326" s="29" t="inlineStr">
         <is>
-          <t>Dow</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="E326" s="29" t="inlineStr">
@@ -34786,17 +34786,17 @@
       </c>
       <c r="C327" s="30" t="inlineStr">
         <is>
-          <t>FCX</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="D327" s="29" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>Comfort Systems</t>
         </is>
       </c>
       <c r="E327" s="29" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F327" s="29" t="inlineStr"/>
@@ -34817,12 +34817,12 @@
       </c>
       <c r="C328" s="30" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="D328" s="29" t="inlineStr">
         <is>
-          <t>Comfort Systems</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="E328" s="29" t="inlineStr">
@@ -34848,17 +34848,17 @@
       </c>
       <c r="C329" s="30" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="D329" s="29" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="E329" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F329" s="29" t="inlineStr"/>
@@ -34879,17 +34879,17 @@
       </c>
       <c r="C330" s="30" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>KNSL</t>
         </is>
       </c>
       <c r="D330" s="29" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Kinsale Capital</t>
         </is>
       </c>
       <c r="E330" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F330" s="29" t="inlineStr"/>
@@ -34910,17 +34910,17 @@
       </c>
       <c r="C331" s="30" t="inlineStr">
         <is>
-          <t>KNSL</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="D331" s="29" t="inlineStr">
         <is>
-          <t>Kinsale Capital</t>
+          <t>Pool Corp</t>
         </is>
       </c>
       <c r="E331" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="F331" s="29" t="inlineStr"/>
@@ -34941,17 +34941,17 @@
       </c>
       <c r="C332" s="30" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>ROP</t>
         </is>
       </c>
       <c r="D332" s="29" t="inlineStr">
         <is>
-          <t>Pool Corp</t>
+          <t>Roper Technologies</t>
         </is>
       </c>
       <c r="E332" s="29" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F332" s="29" t="inlineStr"/>
@@ -34972,17 +34972,17 @@
       </c>
       <c r="C333" s="30" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="D333" s="29" t="inlineStr">
         <is>
-          <t>Roper Technologies</t>
+          <t>RTX Corp</t>
         </is>
       </c>
       <c r="E333" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F333" s="29" t="inlineStr"/>
@@ -36956,12 +36956,12 @@
       </c>
       <c r="C397" s="30" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>TYL</t>
         </is>
       </c>
       <c r="D397" s="29" t="inlineStr">
         <is>
-          <t>TTM Technologies</t>
+          <t>Tyler Technologies</t>
         </is>
       </c>
       <c r="E397" s="29" t="inlineStr">
@@ -36987,17 +36987,17 @@
       </c>
       <c r="C398" s="30" t="inlineStr">
         <is>
-          <t>TYL</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="D398" s="29" t="inlineStr">
         <is>
-          <t>Tyler Technologies</t>
+          <t>Verizon</t>
         </is>
       </c>
       <c r="E398" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="F398" s="29" t="inlineStr"/>
@@ -37018,17 +37018,17 @@
       </c>
       <c r="C399" s="30" t="inlineStr">
         <is>
-          <t>VZ</t>
+          <t>WSO</t>
         </is>
       </c>
       <c r="D399" s="29" t="inlineStr">
         <is>
-          <t>Verizon</t>
+          <t>Watsco</t>
         </is>
       </c>
       <c r="E399" s="29" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F399" s="29" t="inlineStr"/>
@@ -37040,26 +37040,26 @@
     </row>
     <row r="400">
       <c r="A400" s="28" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B400" s="29" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C400" s="30" t="inlineStr">
         <is>
-          <t>WSO</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="D400" s="29" t="inlineStr">
         <is>
-          <t>Watsco</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="E400" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F400" s="29" t="inlineStr"/>
@@ -37080,12 +37080,12 @@
       </c>
       <c r="C401" s="30" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ALGM</t>
         </is>
       </c>
       <c r="D401" s="29" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Allegro MicroSystems</t>
         </is>
       </c>
       <c r="E401" s="29" t="inlineStr">
@@ -37111,17 +37111,17 @@
       </c>
       <c r="C402" s="30" t="inlineStr">
         <is>
-          <t>ALGM</t>
+          <t>AME</t>
         </is>
       </c>
       <c r="D402" s="29" t="inlineStr">
         <is>
-          <t>Allegro MicroSystems</t>
+          <t>AMETEK</t>
         </is>
       </c>
       <c r="E402" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F402" s="29" t="inlineStr"/>
@@ -37142,17 +37142,17 @@
       </c>
       <c r="C403" s="30" t="inlineStr">
         <is>
-          <t>AME</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="D403" s="29" t="inlineStr">
         <is>
-          <t>AMETEK</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="E403" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="F403" s="29" t="inlineStr"/>
@@ -37173,17 +37173,17 @@
       </c>
       <c r="C404" s="30" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="D404" s="29" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>ASE Technology</t>
         </is>
       </c>
       <c r="E404" s="29" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F404" s="29" t="inlineStr"/>
@@ -37204,17 +37204,17 @@
       </c>
       <c r="C405" s="30" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="D405" s="29" t="inlineStr">
         <is>
-          <t>ASE Technology</t>
+          <t>CMS Energy</t>
         </is>
       </c>
       <c r="E405" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="F405" s="29" t="inlineStr"/>
@@ -37235,17 +37235,17 @@
       </c>
       <c r="C406" s="30" t="inlineStr">
         <is>
-          <t>CMS</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="D406" s="29" t="inlineStr">
         <is>
-          <t>CMS Energy</t>
+          <t>DexCom</t>
         </is>
       </c>
       <c r="E406" s="29" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F406" s="29" t="inlineStr"/>
@@ -37266,17 +37266,17 @@
       </c>
       <c r="C407" s="30" t="inlineStr">
         <is>
-          <t>DXCM</t>
+          <t>EPD</t>
         </is>
       </c>
       <c r="D407" s="29" t="inlineStr">
         <is>
-          <t>DexCom</t>
+          <t>Enterprise Products</t>
         </is>
       </c>
       <c r="E407" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F407" s="29" t="inlineStr"/>
@@ -37297,17 +37297,17 @@
       </c>
       <c r="C408" s="30" t="inlineStr">
         <is>
-          <t>EPD</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="D408" s="29" t="inlineStr">
         <is>
-          <t>Enterprise Products</t>
+          <t>Gilead Sciences</t>
         </is>
       </c>
       <c r="E408" s="29" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F408" s="29" t="inlineStr"/>
@@ -37328,17 +37328,17 @@
       </c>
       <c r="C409" s="30" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>HLI</t>
         </is>
       </c>
       <c r="D409" s="29" t="inlineStr">
         <is>
-          <t>Gilead Sciences</t>
+          <t>Houlihan Lokey</t>
         </is>
       </c>
       <c r="E409" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F409" s="29" t="inlineStr"/>
@@ -37359,12 +37359,12 @@
       </c>
       <c r="C410" s="30" t="inlineStr">
         <is>
-          <t>HLI</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D410" s="29" t="inlineStr">
         <is>
-          <t>Houlihan Lokey</t>
+          <t>Intercontinental Ex</t>
         </is>
       </c>
       <c r="E410" s="29" t="inlineStr">
@@ -37390,17 +37390,17 @@
       </c>
       <c r="C411" s="30" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>LHX</t>
         </is>
       </c>
       <c r="D411" s="29" t="inlineStr">
         <is>
-          <t>Intercontinental Ex</t>
+          <t>L3Harris</t>
         </is>
       </c>
       <c r="E411" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F411" s="29" t="inlineStr"/>
@@ -37421,17 +37421,17 @@
       </c>
       <c r="C412" s="30" t="inlineStr">
         <is>
-          <t>LHX</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="D412" s="29" t="inlineStr">
         <is>
-          <t>L3Harris</t>
+          <t>Eli Lilly</t>
         </is>
       </c>
       <c r="E412" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F412" s="29" t="inlineStr"/>
@@ -37452,17 +37452,17 @@
       </c>
       <c r="C413" s="30" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="D413" s="29" t="inlineStr">
         <is>
-          <t>Eli Lilly</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="E413" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F413" s="29" t="inlineStr"/>
@@ -37483,17 +37483,17 @@
       </c>
       <c r="C414" s="30" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="D414" s="29" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Altria</t>
         </is>
       </c>
       <c r="E414" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="F414" s="29" t="inlineStr"/>
@@ -37514,17 +37514,17 @@
       </c>
       <c r="C415" s="30" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="D415" s="29" t="inlineStr">
         <is>
-          <t>Altria</t>
+          <t>Monolithic Power</t>
         </is>
       </c>
       <c r="E415" s="29" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F415" s="29" t="inlineStr"/>
@@ -37545,17 +37545,17 @@
       </c>
       <c r="C416" s="30" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="D416" s="29" t="inlineStr">
         <is>
-          <t>Monolithic Power</t>
+          <t>Merck</t>
         </is>
       </c>
       <c r="E416" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F416" s="29" t="inlineStr"/>
@@ -37576,17 +37576,17 @@
       </c>
       <c r="C417" s="30" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>MSI</t>
         </is>
       </c>
       <c r="D417" s="29" t="inlineStr">
         <is>
-          <t>Merck</t>
+          <t>Motorola Solutions</t>
         </is>
       </c>
       <c r="E417" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F417" s="29" t="inlineStr"/>
@@ -37607,12 +37607,12 @@
       </c>
       <c r="C418" s="30" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="D418" s="29" t="inlineStr">
         <is>
-          <t>Motorola Solutions</t>
+          <t>Strategy (MicroStrategy)</t>
         </is>
       </c>
       <c r="E418" s="29" t="inlineStr">
@@ -37638,12 +37638,12 @@
       </c>
       <c r="C419" s="30" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>NET</t>
         </is>
       </c>
       <c r="D419" s="29" t="inlineStr">
         <is>
-          <t>Strategy (MicroStrategy)</t>
+          <t>Cloudflare</t>
         </is>
       </c>
       <c r="E419" s="29" t="inlineStr">
@@ -37669,17 +37669,17 @@
       </c>
       <c r="C420" s="30" t="inlineStr">
         <is>
-          <t>NET</t>
+          <t>RIOT</t>
         </is>
       </c>
       <c r="D420" s="29" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
+          <t>Riot Platforms</t>
         </is>
       </c>
       <c r="E420" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F420" s="29" t="inlineStr"/>
@@ -37700,17 +37700,17 @@
       </c>
       <c r="C421" s="30" t="inlineStr">
         <is>
-          <t>RIOT</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="D421" s="29" t="inlineStr">
         <is>
-          <t>Riot Platforms</t>
+          <t>Southern Company</t>
         </is>
       </c>
       <c r="E421" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="F421" s="29" t="inlineStr"/>
@@ -37731,17 +37731,17 @@
       </c>
       <c r="C422" s="30" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>SPGI</t>
         </is>
       </c>
       <c r="D422" s="29" t="inlineStr">
         <is>
-          <t>Southern Company</t>
+          <t>S&amp;P Global</t>
         </is>
       </c>
       <c r="E422" s="29" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F422" s="29" t="inlineStr"/>
@@ -37762,17 +37762,17 @@
       </c>
       <c r="C423" s="30" t="inlineStr">
         <is>
-          <t>SPGI</t>
+          <t>SYK</t>
         </is>
       </c>
       <c r="D423" s="29" t="inlineStr">
         <is>
-          <t>S&amp;P Global</t>
+          <t>Stryker</t>
         </is>
       </c>
       <c r="E423" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F423" s="29" t="inlineStr"/>
@@ -37793,17 +37793,17 @@
       </c>
       <c r="C424" s="30" t="inlineStr">
         <is>
-          <t>SYK</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="D424" s="29" t="inlineStr">
         <is>
-          <t>Stryker</t>
+          <t>Trane Technologies</t>
         </is>
       </c>
       <c r="E424" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F424" s="29" t="inlineStr"/>
@@ -37824,17 +37824,17 @@
       </c>
       <c r="C425" s="30" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>TWLO</t>
         </is>
       </c>
       <c r="D425" s="29" t="inlineStr">
         <is>
-          <t>Trane Technologies</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="E425" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F425" s="29" t="inlineStr"/>
@@ -37855,12 +37855,12 @@
       </c>
       <c r="C426" s="30" t="inlineStr">
         <is>
-          <t>TWLO</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="D426" s="29" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Western Digital</t>
         </is>
       </c>
       <c r="E426" s="29" t="inlineStr">
@@ -37886,17 +37886,17 @@
       </c>
       <c r="C427" s="30" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>WEC</t>
         </is>
       </c>
       <c r="D427" s="29" t="inlineStr">
         <is>
-          <t>Western Digital</t>
+          <t>WEC Energy</t>
         </is>
       </c>
       <c r="E427" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="F427" s="29" t="inlineStr"/>
@@ -37908,26 +37908,26 @@
     </row>
     <row r="428">
       <c r="A428" s="28" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="B428" s="29" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C428" s="30" t="inlineStr">
         <is>
-          <t>WEC</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="D428" s="29" t="inlineStr">
         <is>
-          <t>WEC Energy</t>
+          <t>AbbVie</t>
         </is>
       </c>
       <c r="E428" s="29" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F428" s="29" t="inlineStr"/>
@@ -37948,17 +37948,17 @@
       </c>
       <c r="C429" s="30" t="inlineStr">
         <is>
-          <t>ABBV</t>
+          <t>AGCO</t>
         </is>
       </c>
       <c r="D429" s="29" t="inlineStr">
         <is>
-          <t>AbbVie</t>
+          <t>AGCO</t>
         </is>
       </c>
       <c r="E429" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F429" s="29" t="inlineStr"/>
@@ -37979,17 +37979,17 @@
       </c>
       <c r="C430" s="30" t="inlineStr">
         <is>
-          <t>AGCO</t>
+          <t>AON</t>
         </is>
       </c>
       <c r="D430" s="29" t="inlineStr">
         <is>
-          <t>AGCO</t>
+          <t>Aon</t>
         </is>
       </c>
       <c r="E430" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F430" s="29" t="inlineStr"/>
@@ -38010,17 +38010,17 @@
       </c>
       <c r="C431" s="30" t="inlineStr">
         <is>
-          <t>AON</t>
+          <t>CHD</t>
         </is>
       </c>
       <c r="D431" s="29" t="inlineStr">
         <is>
-          <t>Aon</t>
+          <t>Church &amp; Dwight</t>
         </is>
       </c>
       <c r="E431" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="F431" s="29" t="inlineStr"/>
@@ -38041,12 +38041,12 @@
       </c>
       <c r="C432" s="30" t="inlineStr">
         <is>
-          <t>CHD</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="D432" s="29" t="inlineStr">
         <is>
-          <t>Church &amp; Dwight</t>
+          <t>Colgate-Palmolive</t>
         </is>
       </c>
       <c r="E432" s="29" t="inlineStr">
@@ -38072,17 +38072,17 @@
       </c>
       <c r="C433" s="30" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="D433" s="29" t="inlineStr">
         <is>
-          <t>Colgate-Palmolive</t>
+          <t>Chevron</t>
         </is>
       </c>
       <c r="E433" s="29" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F433" s="29" t="inlineStr"/>
@@ -38103,17 +38103,17 @@
       </c>
       <c r="C434" s="30" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>FRT</t>
         </is>
       </c>
       <c r="D434" s="29" t="inlineStr">
         <is>
-          <t>Chevron</t>
+          <t>Federal Realty</t>
         </is>
       </c>
       <c r="E434" s="29" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="F434" s="29" t="inlineStr"/>
@@ -38134,17 +38134,17 @@
       </c>
       <c r="C435" s="30" t="inlineStr">
         <is>
-          <t>FRT</t>
+          <t>GWW</t>
         </is>
       </c>
       <c r="D435" s="29" t="inlineStr">
         <is>
-          <t>Federal Realty</t>
+          <t>W.W. Grainger</t>
         </is>
       </c>
       <c r="E435" s="29" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F435" s="29" t="inlineStr"/>
@@ -38165,17 +38165,17 @@
       </c>
       <c r="C436" s="30" t="inlineStr">
         <is>
-          <t>GWW</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="D436" s="29" t="inlineStr">
         <is>
-          <t>W.W. Grainger</t>
+          <t>Linde</t>
         </is>
       </c>
       <c r="E436" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F436" s="29" t="inlineStr"/>
@@ -38196,17 +38196,17 @@
       </c>
       <c r="C437" s="30" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>RBC</t>
         </is>
       </c>
       <c r="D437" s="29" t="inlineStr">
         <is>
-          <t>Linde</t>
+          <t>RBC Bearings</t>
         </is>
       </c>
       <c r="E437" s="29" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F437" s="29" t="inlineStr"/>
@@ -38227,17 +38227,17 @@
       </c>
       <c r="C438" s="30" t="inlineStr">
         <is>
-          <t>RBC</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="D438" s="29" t="inlineStr">
         <is>
-          <t>RBC Bearings</t>
+          <t>Exxon Mobil</t>
         </is>
       </c>
       <c r="E438" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F438" s="29" t="inlineStr"/>
@@ -38249,21 +38249,21 @@
     </row>
     <row r="439">
       <c r="A439" s="28" t="n">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="B439" s="29" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C439" s="30" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>FANG</t>
         </is>
       </c>
       <c r="D439" s="29" t="inlineStr">
         <is>
-          <t>Exxon Mobil</t>
+          <t>Diamondback Energy</t>
         </is>
       </c>
       <c r="E439" s="29" t="inlineStr">
@@ -38289,17 +38289,17 @@
       </c>
       <c r="C440" s="30" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="D440" s="29" t="inlineStr">
         <is>
-          <t>Diamondback Energy</t>
+          <t>Fabrinet</t>
         </is>
       </c>
       <c r="E440" s="29" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F440" s="29" t="inlineStr"/>
@@ -38320,17 +38320,17 @@
       </c>
       <c r="C441" s="30" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="D441" s="29" t="inlineStr">
         <is>
-          <t>Fabrinet</t>
+          <t>IDEXX Labs</t>
         </is>
       </c>
       <c r="E441" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F441" s="29" t="inlineStr"/>
@@ -38351,17 +38351,17 @@
       </c>
       <c r="C442" s="30" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>O</t>
         </is>
       </c>
       <c r="D442" s="29" t="inlineStr">
         <is>
-          <t>IDEXX Labs</t>
+          <t>Realty Income</t>
         </is>
       </c>
       <c r="E442" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="F442" s="29" t="inlineStr"/>
@@ -38382,17 +38382,17 @@
       </c>
       <c r="C443" s="30" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="D443" s="29" t="inlineStr">
         <is>
-          <t>Realty Income</t>
+          <t>ON Semiconductor</t>
         </is>
       </c>
       <c r="E443" s="29" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F443" s="29" t="inlineStr"/>
@@ -38413,12 +38413,12 @@
       </c>
       <c r="C444" s="30" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="D444" s="29" t="inlineStr">
         <is>
-          <t>ON Semiconductor</t>
+          <t>Palantir</t>
         </is>
       </c>
       <c r="E444" s="29" t="inlineStr">
@@ -38444,12 +38444,12 @@
       </c>
       <c r="C445" s="30" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>SANM</t>
         </is>
       </c>
       <c r="D445" s="29" t="inlineStr">
         <is>
-          <t>Palantir</t>
+          <t>Sanmina</t>
         </is>
       </c>
       <c r="E445" s="29" t="inlineStr">
@@ -38475,17 +38475,17 @@
       </c>
       <c r="C446" s="30" t="inlineStr">
         <is>
-          <t>SANM</t>
+          <t>SPG</t>
         </is>
       </c>
       <c r="D446" s="29" t="inlineStr">
         <is>
-          <t>Sanmina</t>
+          <t>Simon Property</t>
         </is>
       </c>
       <c r="E446" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="F446" s="29" t="inlineStr"/>
@@ -38506,17 +38506,17 @@
       </c>
       <c r="C447" s="30" t="inlineStr">
         <is>
-          <t>SPG</t>
+          <t>VNOM</t>
         </is>
       </c>
       <c r="D447" s="29" t="inlineStr">
         <is>
-          <t>Simon Property</t>
+          <t>Viper Energy</t>
         </is>
       </c>
       <c r="E447" s="29" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F447" s="29" t="inlineStr"/>
@@ -38537,12 +38537,12 @@
       </c>
       <c r="C448" s="30" t="inlineStr">
         <is>
-          <t>VNOM</t>
+          <t>WMB</t>
         </is>
       </c>
       <c r="D448" s="29" t="inlineStr">
         <is>
-          <t>Viper Energy</t>
+          <t>Williams Companies</t>
         </is>
       </c>
       <c r="E448" s="29" t="inlineStr">
@@ -38559,26 +38559,26 @@
     </row>
     <row r="449">
       <c r="A449" s="28" t="n">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="B449" s="29" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="C449" s="30" t="inlineStr">
         <is>
-          <t>WMB</t>
+          <t>ACLS</t>
         </is>
       </c>
       <c r="D449" s="29" t="inlineStr">
         <is>
-          <t>Williams Companies</t>
+          <t>Axcelis</t>
         </is>
       </c>
       <c r="E449" s="29" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F449" s="29" t="inlineStr"/>
@@ -38599,12 +38599,12 @@
       </c>
       <c r="C450" s="30" t="inlineStr">
         <is>
-          <t>ACLS</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="D450" s="29" t="inlineStr">
         <is>
-          <t>Axcelis</t>
+          <t>Advanced Energy</t>
         </is>
       </c>
       <c r="E450" s="29" t="inlineStr">
@@ -38630,17 +38630,17 @@
       </c>
       <c r="C451" s="30" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>AFL</t>
         </is>
       </c>
       <c r="D451" s="29" t="inlineStr">
         <is>
-          <t>Advanced Energy</t>
+          <t>Aflac</t>
         </is>
       </c>
       <c r="E451" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F451" s="29" t="inlineStr"/>
@@ -38661,17 +38661,17 @@
       </c>
       <c r="C452" s="30" t="inlineStr">
         <is>
-          <t>AFL</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="D452" s="29" t="inlineStr">
         <is>
-          <t>Aflac</t>
+          <t>Astera Labs</t>
         </is>
       </c>
       <c r="E452" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F452" s="29" t="inlineStr"/>
@@ -38692,12 +38692,12 @@
       </c>
       <c r="C453" s="30" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="D453" s="29" t="inlineStr">
         <is>
-          <t>Astera Labs</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="E453" s="29" t="inlineStr">
@@ -38723,17 +38723,17 @@
       </c>
       <c r="C454" s="30" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D454" s="29" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="E454" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F454" s="29" t="inlineStr"/>
@@ -38754,17 +38754,17 @@
       </c>
       <c r="C455" s="30" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="D455" s="29" t="inlineStr">
         <is>
-          <t>Amgen</t>
+          <t>Arista Networks</t>
         </is>
       </c>
       <c r="E455" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F455" s="29" t="inlineStr"/>
@@ -38785,17 +38785,17 @@
       </c>
       <c r="C456" s="30" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="D456" s="29" t="inlineStr">
         <is>
-          <t>Arista Networks</t>
+          <t>Broadridge</t>
         </is>
       </c>
       <c r="E456" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F456" s="29" t="inlineStr"/>
@@ -38816,12 +38816,12 @@
       </c>
       <c r="C457" s="30" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="D457" s="29" t="inlineStr">
         <is>
-          <t>Broadridge</t>
+          <t>Eaton</t>
         </is>
       </c>
       <c r="E457" s="29" t="inlineStr">
@@ -38847,17 +38847,17 @@
       </c>
       <c r="C458" s="30" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="D458" s="29" t="inlineStr">
         <is>
-          <t>Eaton</t>
+          <t>Hut 8</t>
         </is>
       </c>
       <c r="E458" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F458" s="29" t="inlineStr"/>
@@ -38878,12 +38878,12 @@
       </c>
       <c r="C459" s="30" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>JKHY</t>
         </is>
       </c>
       <c r="D459" s="29" t="inlineStr">
         <is>
-          <t>Hut 8</t>
+          <t>Jack Henry</t>
         </is>
       </c>
       <c r="E459" s="29" t="inlineStr">
@@ -38909,17 +38909,17 @@
       </c>
       <c r="C460" s="30" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="D460" s="29" t="inlineStr">
         <is>
-          <t>Jack Henry</t>
+          <t>Lumentum</t>
         </is>
       </c>
       <c r="E460" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F460" s="29" t="inlineStr"/>
@@ -38940,17 +38940,17 @@
       </c>
       <c r="C461" s="30" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>MLM</t>
         </is>
       </c>
       <c r="D461" s="29" t="inlineStr">
         <is>
-          <t>Lumentum</t>
+          <t>Martin Marietta</t>
         </is>
       </c>
       <c r="E461" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F461" s="29" t="inlineStr"/>
@@ -38971,17 +38971,17 @@
       </c>
       <c r="C462" s="30" t="inlineStr">
         <is>
-          <t>MLM</t>
+          <t>MTCH</t>
         </is>
       </c>
       <c r="D462" s="29" t="inlineStr">
         <is>
-          <t>Martin Marietta</t>
+          <t>Match Group</t>
         </is>
       </c>
       <c r="E462" s="29" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="F462" s="29" t="inlineStr"/>
@@ -39002,17 +39002,17 @@
       </c>
       <c r="C463" s="30" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="D463" s="29" t="inlineStr">
         <is>
-          <t>Match Group</t>
+          <t>Pfizer</t>
         </is>
       </c>
       <c r="E463" s="29" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F463" s="29" t="inlineStr"/>
@@ -39033,17 +39033,17 @@
       </c>
       <c r="C464" s="30" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="D464" s="29" t="inlineStr">
         <is>
-          <t>Pfizer</t>
+          <t>Super Micro</t>
         </is>
       </c>
       <c r="E464" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F464" s="29" t="inlineStr"/>
@@ -39064,17 +39064,17 @@
       </c>
       <c r="C465" s="30" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>SPOT</t>
         </is>
       </c>
       <c r="D465" s="29" t="inlineStr">
         <is>
-          <t>Super Micro</t>
+          <t>Spotify</t>
         </is>
       </c>
       <c r="E465" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="F465" s="29" t="inlineStr"/>
@@ -39095,17 +39095,17 @@
       </c>
       <c r="C466" s="30" t="inlineStr">
         <is>
-          <t>SPOT</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="D466" s="29" t="inlineStr">
         <is>
-          <t>Spotify</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="E466" s="29" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="F466" s="29" t="inlineStr"/>
@@ -39126,17 +39126,17 @@
       </c>
       <c r="C467" s="30" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>WOLF</t>
         </is>
       </c>
       <c r="D467" s="29" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>Wolfspeed</t>
         </is>
       </c>
       <c r="E467" s="29" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F467" s="29" t="inlineStr"/>
@@ -39157,17 +39157,17 @@
       </c>
       <c r="C468" s="30" t="inlineStr">
         <is>
-          <t>WOLF</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="D468" s="29" t="inlineStr">
         <is>
-          <t>Wolfspeed</t>
+          <t>Zoetis</t>
         </is>
       </c>
       <c r="E468" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F468" s="29" t="inlineStr"/>
@@ -39179,26 +39179,26 @@
     </row>
     <row r="469">
       <c r="A469" s="28" t="n">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="B469" s="29" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="C469" s="30" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="D469" s="29" t="inlineStr">
         <is>
-          <t>Zoetis</t>
+          <t>Arm Holdings</t>
         </is>
       </c>
       <c r="E469" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F469" s="29" t="inlineStr"/>
@@ -39219,17 +39219,17 @@
       </c>
       <c r="C470" s="30" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ATO</t>
         </is>
       </c>
       <c r="D470" s="29" t="inlineStr">
         <is>
-          <t>Arm Holdings</t>
+          <t>Atmos Energy</t>
         </is>
       </c>
       <c r="E470" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="F470" s="29" t="inlineStr"/>
@@ -39250,12 +39250,12 @@
       </c>
       <c r="C471" s="30" t="inlineStr">
         <is>
-          <t>ATO</t>
+          <t>BEPC</t>
         </is>
       </c>
       <c r="D471" s="29" t="inlineStr">
         <is>
-          <t>Atmos Energy</t>
+          <t>Brookfield Renewable</t>
         </is>
       </c>
       <c r="E471" s="29" t="inlineStr">
@@ -39281,17 +39281,17 @@
       </c>
       <c r="C472" s="30" t="inlineStr">
         <is>
-          <t>BEPC</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="D472" s="29" t="inlineStr">
         <is>
-          <t>Brookfield Renewable</t>
+          <t>Coherent</t>
         </is>
       </c>
       <c r="E472" s="29" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F472" s="29" t="inlineStr"/>
@@ -39312,17 +39312,17 @@
       </c>
       <c r="C473" s="30" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D473" s="29" t="inlineStr">
         <is>
-          <t>Coherent</t>
+          <t>Cencora</t>
         </is>
       </c>
       <c r="E473" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F473" s="29" t="inlineStr"/>
@@ -39343,17 +39343,17 @@
       </c>
       <c r="C474" s="30" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>CPAY</t>
         </is>
       </c>
       <c r="D474" s="29" t="inlineStr">
         <is>
-          <t>Cencora</t>
+          <t>Corpay</t>
         </is>
       </c>
       <c r="E474" s="29" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F474" s="29" t="inlineStr"/>
@@ -39374,17 +39374,17 @@
       </c>
       <c r="C475" s="30" t="inlineStr">
         <is>
-          <t>CPAY</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D475" s="29" t="inlineStr">
         <is>
-          <t>Corpay</t>
+          <t>Dynatrace</t>
         </is>
       </c>
       <c r="E475" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F475" s="29" t="inlineStr"/>
@@ -39405,17 +39405,17 @@
       </c>
       <c r="C476" s="30" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>EMR</t>
         </is>
       </c>
       <c r="D476" s="29" t="inlineStr">
         <is>
-          <t>Dynatrace</t>
+          <t>Emerson Electric</t>
         </is>
       </c>
       <c r="E476" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F476" s="29" t="inlineStr"/>
@@ -39436,17 +39436,17 @@
       </c>
       <c r="C477" s="30" t="inlineStr">
         <is>
-          <t>EMR</t>
+          <t>ET</t>
         </is>
       </c>
       <c r="D477" s="29" t="inlineStr">
         <is>
-          <t>Emerson Electric</t>
+          <t>Energy Transfer</t>
         </is>
       </c>
       <c r="E477" s="29" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F477" s="29" t="inlineStr"/>
@@ -39467,17 +39467,17 @@
       </c>
       <c r="C478" s="30" t="inlineStr">
         <is>
-          <t>ET</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="D478" s="29" t="inlineStr">
         <is>
-          <t>Energy Transfer</t>
+          <t>Fortinet</t>
         </is>
       </c>
       <c r="E478" s="29" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F478" s="29" t="inlineStr"/>
@@ -39498,17 +39498,17 @@
       </c>
       <c r="C479" s="30" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="D479" s="29" t="inlineStr">
         <is>
-          <t>Fortinet</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="E479" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F479" s="29" t="inlineStr"/>
@@ -39529,17 +39529,17 @@
       </c>
       <c r="C480" s="30" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="D480" s="29" t="inlineStr">
         <is>
-          <t>Robinhood</t>
+          <t>HubSpot</t>
         </is>
       </c>
       <c r="E480" s="29" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F480" s="29" t="inlineStr"/>
@@ -39560,12 +39560,12 @@
       </c>
       <c r="C481" s="30" t="inlineStr">
         <is>
-          <t>HUBS</t>
+          <t>IONQ</t>
         </is>
       </c>
       <c r="D481" s="29" t="inlineStr">
         <is>
-          <t>HubSpot</t>
+          <t>IonQ</t>
         </is>
       </c>
       <c r="E481" s="29" t="inlineStr">
@@ -39591,17 +39591,17 @@
       </c>
       <c r="C482" s="30" t="inlineStr">
         <is>
-          <t>IONQ</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="D482" s="29" t="inlineStr">
         <is>
-          <t>IonQ</t>
+          <t>McDonald's</t>
         </is>
       </c>
       <c r="E482" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="F482" s="29" t="inlineStr"/>
@@ -39622,17 +39622,17 @@
       </c>
       <c r="C483" s="30" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="D483" s="29" t="inlineStr">
         <is>
-          <t>McDonald's</t>
+          <t>MKS Instruments</t>
         </is>
       </c>
       <c r="E483" s="29" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F483" s="29" t="inlineStr"/>
@@ -39653,12 +39653,12 @@
       </c>
       <c r="C484" s="30" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="D484" s="29" t="inlineStr">
         <is>
-          <t>MKS Instruments</t>
+          <t>Qualcomm</t>
         </is>
       </c>
       <c r="E484" s="29" t="inlineStr">
@@ -39684,17 +39684,17 @@
       </c>
       <c r="C485" s="30" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="D485" s="29" t="inlineStr">
         <is>
-          <t>Qualcomm</t>
+          <t>Sportradar</t>
         </is>
       </c>
       <c r="E485" s="29" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="F485" s="29" t="inlineStr"/>
@@ -39715,17 +39715,17 @@
       </c>
       <c r="C486" s="30" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>TKO</t>
         </is>
       </c>
       <c r="D486" s="29" t="inlineStr">
         <is>
-          <t>Sportradar</t>
+          <t>TKO Group</t>
         </is>
       </c>
       <c r="E486" s="29" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="F486" s="29" t="inlineStr"/>
@@ -39746,17 +39746,17 @@
       </c>
       <c r="C487" s="30" t="inlineStr">
         <is>
-          <t>TKO</t>
+          <t>TRMB</t>
         </is>
       </c>
       <c r="D487" s="29" t="inlineStr">
         <is>
-          <t>TKO Group</t>
+          <t>Trimble</t>
         </is>
       </c>
       <c r="E487" s="29" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="F487" s="29" t="inlineStr"/>
@@ -39777,12 +39777,12 @@
       </c>
       <c r="C488" s="30" t="inlineStr">
         <is>
-          <t>TRMB</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="D488" s="29" t="inlineStr">
         <is>
-          <t>Trimble</t>
+          <t>TTM Technologies</t>
         </is>
       </c>
       <c r="E488" s="29" t="inlineStr">
@@ -43952,7 +43952,7 @@
       <c r="B36" s="38" t="inlineStr">
         <is>
           <t>20
-ADC CB DHR GE GM GPC HAL ISRG KO LMT NFLX OMC PCAR PEGA RTX TXN</t>
+ADC CB DHR GE GM GPC HAL ISRG KO LMT NFLX OMC PCAR PEGA TXN</t>
         </is>
       </c>
       <c r="C36" s="38" t="inlineStr">
@@ -43964,7 +43964,7 @@
       <c r="D36" s="38" t="inlineStr">
         <is>
           <t>22
-BKR BX CBRE DLR DOW FCX FIX HON INTC KNSL POOL ROP TMUS TSCO UNP</t>
+BKR BX CBRE DLR DOW FCX FIX HON INTC KNSL POOL ROP RTX TMUS TSCO UNP</t>
         </is>
       </c>
       <c r="E36" s="38" t="inlineStr">
@@ -44000,7 +44000,7 @@
       <c r="C37" s="38" t="inlineStr">
         <is>
           <t>28
-ADP AWK BA CAT CMG COHU CVS EQIX ETR FORM GOOGL KHC KLAC META MKL MSFT NOW ODFL PI PSA PSX ROL SAN SBUX SUI TEL TTMI TYL VZ WSO</t>
+ADP AWK BA CAT CMG COHU CVS EQIX ETR FORM GOOGL KHC KLAC META MKL MSFT NOW ODFL PI PSA PSX ROL SAN SBUX SUI TEL TYL VZ WSO</t>
         </is>
       </c>
       <c r="D37" s="38" t="inlineStr">
@@ -44095,7 +44095,7 @@
       <c r="C43" s="38" t="inlineStr">
         <is>
           <t>4
-ARM ATO BEPC COHR COR CPAY DT EMR ET FTNT HOOD HUBS IONQ MCD MKSI QCOM SRAD TKO TRMB U</t>
+ARM ATO BEPC COHR COR CPAY DT EMR ET FTNT HOOD HUBS IONQ MCD MKSI QCOM SRAD TKO TRMB TTMI U</t>
         </is>
       </c>
       <c r="D43" s="38" t="inlineStr">

</xml_diff>